<commit_message>
fix(fuzzing): khac phuc loi UnicodeDecodeError cp1252 tren Windows cho fuzz harness va cap nhat log
</commit_message>
<xml_diff>
--- a/docs/06_Dynamic_Fuzzing/fuzzing_campaigns.xlsx
+++ b/docs/06_Dynamic_Fuzzing/fuzzing_campaigns.xlsx
@@ -543,12 +543,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>19.87</t>
+          <t>20.97</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>50.3</t>
+          <t>47.7</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">

</xml_diff>

<commit_message>
feat(evident): bo sung harness wrapper, anh minh chung audit v1 va cap nhat ket qua dynamic fuzzing
</commit_message>
<xml_diff>
--- a/docs/06_Dynamic_Fuzzing/fuzzing_campaigns.xlsx
+++ b/docs/06_Dynamic_Fuzzing/fuzzing_campaigns.xlsx
@@ -543,12 +543,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>19.00</t>
+          <t>26.35</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>52.6</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">

</xml_diff>